<commit_message>
Minor renaming figures, tables
</commit_message>
<xml_diff>
--- a/Output/tableS1.xlsx
+++ b/Output/tableS1.xlsx
@@ -351,13 +351,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>types</t>
+          <t>factor</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -367,25 +367,15 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>p</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>z</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>lower</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>upper</t>
         </is>
@@ -394,126 +384,229 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>raceBlack</t>
         </is>
       </c>
       <c r="B2">
-        <v>0.001547532387689908</v>
+        <v>0.02098596272796704</v>
       </c>
       <c r="C2">
-        <v>0.003011951727606107</v>
+        <v>0.1444128361854471</v>
       </c>
       <c r="D2">
-        <v>0.5137972078058114</v>
+        <v>-0.00719507488308185</v>
       </c>
       <c r="E2">
-        <v>0.6073937803051694</v>
-      </c>
-      <c r="F2">
-        <v>-0.004355784521591256</v>
-      </c>
-      <c r="G2">
-        <v>0.007450849296971072</v>
+        <v>0.04916700033901594</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>raceHispan</t>
         </is>
       </c>
       <c r="B3">
-        <v>0.003287889403810728</v>
+        <v>0.01853957447406557</v>
       </c>
       <c r="C3">
-        <v>0.00269797664382722</v>
+        <v>0.1846763421092724</v>
       </c>
       <c r="D3">
-        <v>1.218650061828069</v>
+        <v>-0.008853626351854472</v>
       </c>
       <c r="E3">
-        <v>0.2229770394612888</v>
-      </c>
-      <c r="F3">
-        <v>-0.00200004764922087</v>
-      </c>
-      <c r="G3">
-        <v>0.008575826456842326</v>
+        <v>0.04593277529998562</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>125%</t>
+          <t>raceBlack</t>
         </is>
       </c>
       <c r="B4">
-        <v>0.006395028036355884</v>
+        <v>0.02091654159277542</v>
       </c>
       <c r="C4">
-        <v>0.003293361842784922</v>
+        <v>0.0001905644006287766</v>
       </c>
       <c r="D4">
-        <v>1.941793322943264</v>
+        <v>0.009929301827608383</v>
       </c>
       <c r="E4">
-        <v>0.05216212553203638</v>
-      </c>
-      <c r="F4">
-        <v>-5.984256356102516E-05</v>
-      </c>
-      <c r="G4">
-        <v>0.01284989863627279</v>
+        <v>0.03190378135794246</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>150%</t>
+          <t>raceHispan</t>
         </is>
       </c>
       <c r="B5">
-        <v>0.01138220767810092</v>
+        <v>0.03286528498763408</v>
       </c>
       <c r="C5">
-        <v>0.0036449879526175</v>
+        <v>2.16593578452203E-11</v>
       </c>
       <c r="D5">
-        <v>3.122701042105573</v>
+        <v>0.02324306282389042</v>
       </c>
       <c r="E5">
-        <v>0.001791996710039601</v>
-      </c>
-      <c r="F5">
-        <v>0.004238162566888235</v>
-      </c>
-      <c r="G5">
-        <v>0.01852625278931361</v>
+        <v>0.04248750715137774</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>200%</t>
+          <t>raceBlack</t>
         </is>
       </c>
       <c r="B6">
-        <v>0.01141152867328361</v>
+        <v>-0.004887461361262132</v>
       </c>
       <c r="C6">
-        <v>0.004303403338639504</v>
+        <v>0.7216430493930357</v>
       </c>
       <c r="D6">
-        <v>2.651745089943462</v>
+        <v>-0.03177554099257027</v>
       </c>
       <c r="E6">
-        <v>0.00800769721905017</v>
-      </c>
-      <c r="F6">
-        <v>0.002977013118600755</v>
-      </c>
-      <c r="G6">
-        <v>0.01984604422796646</v>
+        <v>0.02200061827004601</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>raceHispan</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>0.01794432420143629</v>
+      </c>
+      <c r="C7">
+        <v>0.1672922401943286</v>
+      </c>
+      <c r="D7">
+        <v>-0.007523691061596817</v>
+      </c>
+      <c r="E7">
+        <v>0.04341233946446939</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>raceBlack</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>0.006489558872915246</v>
+      </c>
+      <c r="C8">
+        <v>0.7494403281029609</v>
+      </c>
+      <c r="D8">
+        <v>-0.03333574093818088</v>
+      </c>
+      <c r="E8">
+        <v>0.04631485868401138</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>raceHispan</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>0.02629791907149458</v>
+      </c>
+      <c r="C9">
+        <v>0.2063238438304791</v>
+      </c>
+      <c r="D9">
+        <v>-0.01448818318615117</v>
+      </c>
+      <c r="E9">
+        <v>0.06708402132914032</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>raceBlack</t>
+        </is>
+      </c>
+      <c r="B10">
+        <v>0.01507714464221724</v>
+      </c>
+      <c r="C10">
+        <v>0.1951426050945523</v>
+      </c>
+      <c r="D10">
+        <v>-0.007732825774645624</v>
+      </c>
+      <c r="E10">
+        <v>0.0378871150590801</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>raceHispan</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>0.01474658975654985</v>
+      </c>
+      <c r="C11">
+        <v>0.2231979514887684</v>
+      </c>
+      <c r="D11">
+        <v>-0.008981784588315332</v>
+      </c>
+      <c r="E11">
+        <v>0.03847496410141502</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>raceBlack</t>
+        </is>
+      </c>
+      <c r="B12">
+        <v>0.05226987291991244</v>
+      </c>
+      <c r="C12">
+        <v>9.555743860594524E-21</v>
+      </c>
+      <c r="D12">
+        <v>0.0413022424558122</v>
+      </c>
+      <c r="E12">
+        <v>0.06323750338401268</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>raceHispan</t>
+        </is>
+      </c>
+      <c r="B13">
+        <v>0.06621745406785411</v>
+      </c>
+      <c r="C13">
+        <v>2.533413209582664E-27</v>
+      </c>
+      <c r="D13">
+        <v>0.05423162517577045</v>
+      </c>
+      <c r="E13">
+        <v>0.07820328295993775</v>
       </c>
     </row>
   </sheetData>

</xml_diff>